<commit_message>
feat: add TP list view and dashboard components
- Implemented `TpListView` for displaying transformer points with filters and a form for adding new TP.
- Created `widgets.tsx` for dashboard KPI cards, donut charts, loss bars, and ranking lists.
- Added `PageTabs` component for navigation within pages using URL parameters.
- Developed `dashboard.ts` to aggregate and compute data for the dashboard, including energy consumption and consumer statistics.
- Introduced `tp-dashboard.ts` for TP-specific dashboard data, including readings, consumer counts, and tariff zones.
</commit_message>
<xml_diff>
--- a/.claude/docs/umumiy_hisobot.xlsx
+++ b/.claude/docs/umumiy_hisobot.xlsx
@@ -43,7 +43,7 @@
     <t>Elektr oqimi</t>
   </si>
   <si>
-    <t>Texnoligik yo'qotish 12%</t>
+    <t>Texnoligik yo'qotish 12% koefitsiyent</t>
   </si>
   <si>
     <t>Tijoriy yo'qotish</t>
@@ -255,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -264,6 +264,9 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
@@ -290,7 +293,9 @@
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -303,10 +308,14 @@
     <xf borderId="1" fillId="3" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="5" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="1" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
@@ -535,7 +544,7 @@
     <col customWidth="1" min="9" max="9" width="15.14"/>
     <col customWidth="1" min="10" max="10" width="10.86"/>
     <col customWidth="1" min="11" max="11" width="11.43"/>
-    <col customWidth="1" min="12" max="12" width="8.71"/>
+    <col customWidth="1" min="12" max="12" width="10.29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,7 +581,7 @@
       <c r="J3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="L3" s="2" t="s">
@@ -582,432 +591,438 @@
     <row r="4">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="4"/>
+      <c r="E4" s="5"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="9"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="10"/>
     </row>
     <row r="5">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <v>1290.0</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <v>1295.0</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="7">
         <f t="shared" ref="G5:G9" si="1">+F5-E5</f>
         <v>5</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="7">
         <f t="shared" ref="I5:I9" si="2">+H5*G5</f>
         <v>20000</v>
       </c>
-      <c r="J5" s="12">
-        <v>20000.0</v>
-      </c>
-      <c r="K5" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="L5" s="14">
-        <v>0.0</v>
-      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="15"/>
     </row>
     <row r="6">
-      <c r="A6" s="10"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="10" t="s">
+      <c r="A6" s="11"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="7">
         <v>9194.0</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="7">
         <f t="shared" si="1"/>
         <v>242</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="7">
         <f t="shared" si="2"/>
         <v>726000</v>
       </c>
-      <c r="J6" s="12"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="14"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="15"/>
     </row>
     <row r="7">
-      <c r="A7" s="10"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="10" t="s">
+      <c r="A7" s="11"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="7">
         <v>10926.0</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="7">
         <f t="shared" si="1"/>
         <v>135</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="7">
         <f t="shared" si="2"/>
         <v>270000</v>
       </c>
-      <c r="J7" s="12"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="14"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="15"/>
     </row>
     <row r="8">
-      <c r="A8" s="10"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="10" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="7">
         <v>3009.0</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="7">
         <f t="shared" si="1"/>
         <v>137</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="7">
         <f t="shared" si="2"/>
         <v>274000</v>
       </c>
-      <c r="J8" s="12"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="14"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="15"/>
     </row>
     <row r="9">
-      <c r="A9" s="10"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="10" t="s">
+      <c r="A9" s="11"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="7">
         <v>845.0</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="7">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="7">
         <f t="shared" si="2"/>
         <v>41000</v>
       </c>
-      <c r="J9" s="12"/>
-      <c r="L9" s="14"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="15"/>
     </row>
     <row r="10">
-      <c r="A10" s="10"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="18">
+      <c r="D10" s="14"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="19">
         <f>SUM(I5:I9)</f>
         <v>1331000</v>
       </c>
-      <c r="J10" s="12"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="14"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="15"/>
     </row>
     <row r="11">
-      <c r="A11" s="10"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="3" t="s">
+      <c r="A11" s="11"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6" t="s">
+      <c r="D11" s="11"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="12"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="14"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="15"/>
     </row>
     <row r="12">
-      <c r="A12" s="10"/>
-      <c r="B12" s="15"/>
-      <c r="D12" s="10" t="s">
+      <c r="A12" s="11"/>
+      <c r="B12" s="16"/>
+      <c r="D12" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="7">
         <v>28325.0</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="7">
         <f t="shared" ref="G12:G17" si="3">+F12-E12</f>
         <v>144</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="19">
+      <c r="I12" s="21">
         <f t="shared" ref="I12:I17" si="4">+H12*G12</f>
         <v>432000</v>
       </c>
-      <c r="J12" s="12">
+      <c r="J12" s="20">
         <v>317911.8</v>
       </c>
-      <c r="K12" s="13">
-        <f t="shared" ref="K12:K18" si="5">+I12*12/100</f>
+      <c r="K12" s="14">
+        <f t="shared" ref="K12:K17" si="5">+I12*12/100</f>
         <v>51840</v>
       </c>
-      <c r="L12" s="20">
-        <f t="shared" ref="L12:L18" si="6">+I12-J12-K12</f>
+      <c r="L12" s="22">
+        <f t="shared" ref="L12:L17" si="6">+I12-J12-K12</f>
         <v>62248.2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="10" t="s">
+      <c r="A13" s="11"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="7">
         <v>8550.0</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="7">
         <f t="shared" si="3"/>
         <v>100</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="7">
         <f t="shared" si="4"/>
         <v>200000</v>
       </c>
-      <c r="J13" s="12">
-        <v>163362.0</v>
-      </c>
-      <c r="K13" s="13">
+      <c r="J13" s="13">
+        <v>155565.7</v>
+      </c>
+      <c r="K13" s="14">
         <f t="shared" si="5"/>
         <v>24000</v>
       </c>
-      <c r="L13" s="20">
+      <c r="L13" s="22">
         <f t="shared" si="6"/>
-        <v>12638</v>
+        <v>20434.3</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="10"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="10" t="s">
+      <c r="A14" s="11"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="6">
-        <v>18707.0</v>
-      </c>
-      <c r="G14" s="6">
+      <c r="F14" s="23">
+        <v>18607.0</v>
+      </c>
+      <c r="G14" s="7">
         <f t="shared" si="3"/>
-        <v>237</v>
-      </c>
-      <c r="H14" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I14" s="7">
         <f t="shared" si="4"/>
-        <v>1422000</v>
-      </c>
-      <c r="J14" s="12"/>
-      <c r="K14" s="13">
+        <v>822000</v>
+      </c>
+      <c r="J14" s="13">
+        <v>565384.9</v>
+      </c>
+      <c r="K14" s="14">
         <f t="shared" si="5"/>
-        <v>170640</v>
-      </c>
-      <c r="L14" s="20">
+        <v>98640</v>
+      </c>
+      <c r="L14" s="22">
         <f t="shared" si="6"/>
-        <v>1251360</v>
+        <v>157975.1</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="10"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="10" t="s">
+      <c r="A15" s="11"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="7">
         <v>7451.0</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="7">
         <f t="shared" si="3"/>
         <v>139</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="7">
         <f t="shared" si="4"/>
         <v>278000</v>
       </c>
-      <c r="J15" s="12"/>
-      <c r="K15" s="13">
+      <c r="J15" s="13">
+        <v>237989.3</v>
+      </c>
+      <c r="K15" s="14">
         <f t="shared" si="5"/>
         <v>33360</v>
       </c>
-      <c r="L15" s="20">
+      <c r="L15" s="22">
         <f t="shared" si="6"/>
-        <v>244640</v>
+        <v>6650.7</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="10"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="10" t="s">
+      <c r="A16" s="11"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="7">
         <v>17594.0</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="7">
         <f t="shared" si="3"/>
         <v>71</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="7">
         <f t="shared" si="4"/>
         <v>213000</v>
       </c>
-      <c r="J16" s="12"/>
-      <c r="K16" s="13">
+      <c r="J16" s="13">
+        <v>155987.9</v>
+      </c>
+      <c r="K16" s="14">
         <f t="shared" si="5"/>
         <v>25560</v>
       </c>
-      <c r="L16" s="20">
+      <c r="L16" s="22">
         <f t="shared" si="6"/>
-        <v>187440</v>
+        <v>31452.1</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="10"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="10" t="s">
+      <c r="A17" s="11"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="6">
-        <v>19989.0</v>
-      </c>
-      <c r="G17" s="6">
+      <c r="F17" s="23">
+        <v>20112.0</v>
+      </c>
+      <c r="G17" s="7">
         <f t="shared" si="3"/>
-        <v>139</v>
-      </c>
-      <c r="H17" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="H17" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="7">
         <f t="shared" si="4"/>
-        <v>556000</v>
-      </c>
-      <c r="J17" s="12"/>
-      <c r="K17" s="13">
+        <v>1048000</v>
+      </c>
+      <c r="J17" s="13">
+        <v>683812.3</v>
+      </c>
+      <c r="K17" s="14">
         <f t="shared" si="5"/>
-        <v>66720</v>
-      </c>
-      <c r="L17" s="20">
+        <v>125760</v>
+      </c>
+      <c r="L17" s="22">
         <f t="shared" si="6"/>
-        <v>489280</v>
+        <v>238427.7</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="13" t="s">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="22">
+      <c r="D18" s="14"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="25">
         <f>SUM(I11:I17)</f>
-        <v>3101000</v>
-      </c>
-      <c r="J18" s="12"/>
-      <c r="K18" s="13">
-        <f t="shared" si="5"/>
-        <v>372120</v>
-      </c>
-      <c r="L18" s="20">
-        <f t="shared" si="6"/>
-        <v>2728880</v>
+        <v>2993000</v>
+      </c>
+      <c r="J18" s="20">
+        <f>J12+J13+J14+J14+J15+J16+J17</f>
+        <v>2682036.8</v>
+      </c>
+      <c r="K18" s="14">
+        <f t="shared" ref="K18:L18" si="7">SUM(K12:K17)</f>
+        <v>359160</v>
+      </c>
+      <c r="L18" s="22">
+        <f t="shared" si="7"/>
+        <v>517188.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>